<commit_message>
Add verified breseq records and complete EcoCyc exports
</commit_message>
<xml_diff>
--- a/working/source-data/Supplementary Table 4.xlsx
+++ b/working/source-data/Supplementary Table 4.xlsx
@@ -655,6 +655,21 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Muhammed Sadik Yildiz</author>
+  </authors>
+  <commentList>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>All 133 rows from the matching original EcoCyc export are retained. The first 19 match the original workbook; rows 21–134 restore the remaining results. Exported P-values extend to &lt;0.1, not all &lt;0.05. See data/single-cell/enrichment/README.md.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -66506,7 +66521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35.5703125" customWidth="1" min="10" max="10"/>
@@ -67075,8 +67090,1714 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>GTPase activity</t>
+        </is>
+      </c>
+      <c r="K21" s="1" t="n">
+        <v>0.0014163393</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>tufB // rplJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>translation regulator activity</t>
+        </is>
+      </c>
+      <c r="K22" s="1" t="n">
+        <v>0.0016187794</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>tufB // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>membraneless organelle</t>
+        </is>
+      </c>
+      <c r="K23" s="1" t="n">
+        <v>0.0017255478</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>rplJ // rplV // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>organelle</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>0.0017645087</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>rplJ // rplV // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>membraneless organelle assembly</t>
+        </is>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>0.001946873</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>rplV // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>organelle assembly</t>
+        </is>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>0.001946873</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>rplV // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>mRNA pseudouridine synthesis</t>
+        </is>
+      </c>
+      <c r="K27" s="1" t="n">
+        <v>0.0020089287</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>tRNA pseudouridine(55) synthase activity</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>0.0020089287</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>mRNA modification</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>0.0020089287</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>RNA-binding transcription regulator activity</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>0.0020089287</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>negative regulation of translation</t>
+        </is>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>0.002062711</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>rplD // rplJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>negative regulation of protein metabolic process</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>0.00268998</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>rplD // rplJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>nucleic acid binding</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>0.0027532505</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>rplJ // truB // rplV // cspG // rplD // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>response to chemical</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>0.0030881355</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>efeO // rplV // rplD // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>dksA</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>0.003320052</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>rplD // rplV // rplJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>response to stimulus</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>0.0038179967</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>efeO // phoR // rplV // cspG // rplD // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>tRNA folding</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>0.004014269</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>PhoRB Two-Component Signal Transduction System, phosphate-dependent</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>0.004014269</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>negative regulation of cytoplasmic translation</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>0.0060160267</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>guanyl-nucleotide exchange factor complex</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>0.0060160267</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>cytosolic ribosome assembly</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>0.0060160267</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>rplV</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>alpA</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>0.0060160267</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>assembly of large subunit precursor of preribosome</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>0.0060160267</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>rplV</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>endoribonuclease inhibitor activity</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>0.008014208</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>ribonuclease inhibitor activity</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>0.008014208</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>nuclease inhibitor activity</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>0.008014208</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>regulation of translation</t>
+        </is>
+      </c>
+      <c r="K47" s="1" t="n">
+        <v>0.009953327999999999</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>rplD // rplJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>organelle organization</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="n">
+        <v>0.009953327999999999</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>rplV // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>RNA folding</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>0.010008818</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>macromolecule biosynthetic process</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>0.010408023</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>rplJ // rplV // rplD // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>tRNA pseudouridine synthesis</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>0.011999861</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>DNA-templated transcription termination</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>0.011999861</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>rplA</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>0.011999861</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>rplJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>regulation of cytoplasmic translation</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>0.011999861</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>tRNA pseudouridine synthase activity</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>0.011999861</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>organic cyclic compound binding</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>0.013516291</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>rplJ // truB // phoR // rplV // cspG // rplD // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>molecular function regulator activity</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>0.013672718</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>rplD // phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>lytic endotransglycosylase activity</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="n">
+        <v>0.013987345</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>mltD</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>regulation of gene expression</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>0.014491825</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // cspG // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>negative regulation of gene expression</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>0.014538327</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>rplD // rplJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>regulation of protein metabolic process</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>0.014538327</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>rplD // rplJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>regulation of macromolecule biosynthetic process</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>0.014686136</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // cspG // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>regulation of biosynthetic process</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>0.01558209</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // cspG // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>translation elongation factor activity</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>0.015971273</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>regulation of macromolecule metabolic process</t>
+        </is>
+      </c>
+      <c r="K65" s="1" t="n">
+        <v>0.017812593</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // cspG // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>carbon-oxygen lyase activity, acting on polysaccharides</t>
+        </is>
+      </c>
+      <c r="K66" s="1" t="n">
+        <v>0.017951652</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>mltD</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>lytic transglycosylase activity</t>
+        </is>
+      </c>
+      <c r="K67" s="1" t="n">
+        <v>0.017951652</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>mltD</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>regulation of metabolic process</t>
+        </is>
+      </c>
+      <c r="K68" s="1" t="n">
+        <v>0.019411284</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // cspG // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>transcriptional attenuation</t>
+        </is>
+      </c>
+      <c r="K69" s="1" t="n">
+        <v>0.019928489</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>translation repressor activity</t>
+        </is>
+      </c>
+      <c r="K70" s="1" t="n">
+        <v>0.019928489</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>post-transcriptional regulation of gene expression</t>
+        </is>
+      </c>
+      <c r="K71" s="1" t="n">
+        <v>0.020901538</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>rplD // rplJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>positive regulation of termination of DNA-templated transcription</t>
+        </is>
+      </c>
+      <c r="K72" s="1" t="n">
+        <v>0.021901788</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>pseudouridine synthase activity</t>
+        </is>
+      </c>
+      <c r="K73" s="1" t="n">
+        <v>0.021901788</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>positive regulation of protein-containing complex disassembly</t>
+        </is>
+      </c>
+      <c r="K74" s="1" t="n">
+        <v>0.021901788</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>cellular response to phosphate starvation</t>
+        </is>
+      </c>
+      <c r="K75" s="1" t="n">
+        <v>0.023871554</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>pseudouridine synthesis</t>
+        </is>
+      </c>
+      <c r="K76" s="1" t="n">
+        <v>0.023871554</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>phosphate ion transport</t>
+        </is>
+      </c>
+      <c r="K77" s="1" t="n">
+        <v>0.025837792</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>translational elongation</t>
+        </is>
+      </c>
+      <c r="K78" s="1" t="n">
+        <v>0.029759713</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>translation factor activity, RNA binding</t>
+        </is>
+      </c>
+      <c r="K79" s="1" t="n">
+        <v>0.037561473</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>peptidoglycan muralytic activity</t>
+        </is>
+      </c>
+      <c r="K80" s="1" t="n">
+        <v>0.037561473</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>mltD</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>mRNA metabolic process</t>
+        </is>
+      </c>
+      <c r="K81" s="1" t="n">
+        <v>0.037561473</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>response to cold</t>
+        </is>
+      </c>
+      <c r="K82" s="1" t="n">
+        <v>0.039503176</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>cspG</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>peptidoglycan recycling I</t>
+        </is>
+      </c>
+      <c r="K83" s="1" t="n">
+        <v>0.039503176</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>mltD</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>regulation of cellular process</t>
+        </is>
+      </c>
+      <c r="K84" s="1" t="n">
+        <v>0.040935636</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // cspG // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>positive regulation of cellular component organization</t>
+        </is>
+      </c>
+      <c r="K85" s="1" t="n">
+        <v>0.0414414</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>cytoplasm</t>
+        </is>
+      </c>
+      <c r="K86" s="1" t="n">
+        <v>0.042138778</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>tufB // cspG // rplV // rplJ // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>phosphoprotein phosphatase activity</t>
+        </is>
+      </c>
+      <c r="K87" s="1" t="n">
+        <v>0.043376144</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>enzyme inhibitor activity</t>
+        </is>
+      </c>
+      <c r="K88" s="1" t="n">
+        <v>0.043376144</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>molecular function inhibitor activity</t>
+        </is>
+      </c>
+      <c r="K89" s="1" t="n">
+        <v>0.045307416</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Degradation/Utilization/Assimilation - Other</t>
+        </is>
+      </c>
+      <c r="K90" s="1" t="n">
+        <v>0.047235224</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>mltD</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>response to UV</t>
+        </is>
+      </c>
+      <c r="K91" s="1" t="n">
+        <v>0.047235224</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>efeO</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>translation regulator activity, nucleic acid binding</t>
+        </is>
+      </c>
+      <c r="K92" s="1" t="n">
+        <v>0.049159568</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>mRNA 5'-UTR binding</t>
+        </is>
+      </c>
+      <c r="K93" s="1" t="n">
+        <v>0.049159568</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>peptidyl-histidine phosphorylation</t>
+        </is>
+      </c>
+      <c r="K94" s="1" t="n">
+        <v>0.051080458</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>peptidyl-histidine modification</t>
+        </is>
+      </c>
+      <c r="K95" s="1" t="n">
+        <v>0.051080458</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>regulation of biological process</t>
+        </is>
+      </c>
+      <c r="K96" s="1" t="n">
+        <v>0.053546924</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // cspG // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>cellular component organization</t>
+        </is>
+      </c>
+      <c r="K97" s="1" t="n">
+        <v>0.05369257</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>mltD // rplV // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>response to toxic substance</t>
+        </is>
+      </c>
+      <c r="K98" s="1" t="n">
+        <v>0.054911893</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>efeO</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>response to light stimulus</t>
+        </is>
+      </c>
+      <c r="K99" s="1" t="n">
+        <v>0.054911893</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>efeO</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>ribonucleoside triphosphate phosphatase activity</t>
+        </is>
+      </c>
+      <c r="K100" s="1" t="n">
+        <v>0.054953042</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>rplJ // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>cellular component organization or biogenesis</t>
+        </is>
+      </c>
+      <c r="K101" s="1" t="n">
+        <v>0.058312554</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>mltD // rplV // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>phosphorelay sensor kinase activity</t>
+        </is>
+      </c>
+      <c r="K102" s="1" t="n">
+        <v>0.05872957</v>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>protein histidine kinase activity</t>
+        </is>
+      </c>
+      <c r="K103" s="1" t="n">
+        <v>0.05872957</v>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>regulation of termination of DNA-templated transcription</t>
+        </is>
+      </c>
+      <c r="K104" s="1" t="n">
+        <v>0.06063326</v>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>biological regulation</t>
+        </is>
+      </c>
+      <c r="K105" s="1" t="n">
+        <v>0.062467877</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // cspG // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>protein autophosphorylation</t>
+        </is>
+      </c>
+      <c r="K106" s="1" t="n">
+        <v>0.062533535</v>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>regulation of protein-containing complex disassembly</t>
+        </is>
+      </c>
+      <c r="K107" s="1" t="n">
+        <v>0.062533535</v>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>macromolecule modification</t>
+        </is>
+      </c>
+      <c r="K108" s="1" t="n">
+        <v>0.06334474</v>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>truB // phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>intramolecular transferase activity</t>
+        </is>
+      </c>
+      <c r="K109" s="1" t="n">
+        <v>0.06443038600000001</v>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>guanosine tetraphosphate binding</t>
+        </is>
+      </c>
+      <c r="K110" s="1" t="n">
+        <v>0.06821386</v>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>phosphotransferase activity, nitrogenous group as acceptor</t>
+        </is>
+      </c>
+      <c r="K111" s="1" t="n">
+        <v>0.06821386</v>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>molecular sensor activity</t>
+        </is>
+      </c>
+      <c r="K112" s="1" t="n">
+        <v>0.07010049</v>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>metabolic process</t>
+        </is>
+      </c>
+      <c r="K113" s="1" t="n">
+        <v>0.07122732</v>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>mltD // rplJ // truB // phoR // rplV // rplD // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>pyrophosphatase activity</t>
+        </is>
+      </c>
+      <c r="K114" s="1" t="n">
+        <v>0.073868304</v>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>rplJ // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>hydrolase activity, acting on acid anhydrides</t>
+        </is>
+      </c>
+      <c r="K115" s="1" t="n">
+        <v>0.07443812</v>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>rplJ // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>hydrolase activity, acting on acid anhydrides, in phosphorus-containing anhydrides</t>
+        </is>
+      </c>
+      <c r="K116" s="1" t="n">
+        <v>0.07443812</v>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>rplJ // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>protein binding</t>
+        </is>
+      </c>
+      <c r="K117" s="1" t="n">
+        <v>0.07547828600000001</v>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // rplV // cspG // rplD // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>regulation of primary metabolic process</t>
+        </is>
+      </c>
+      <c r="K118" s="1" t="n">
+        <v>0.07729772</v>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>rplJ // phoR // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>All-Genes</t>
+        </is>
+      </c>
+      <c r="K119" s="1" t="n">
+        <v>0.07783468</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>arcA</t>
+        </is>
+      </c>
+      <c r="K120" s="1" t="n">
+        <v>0.07788922</v>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>rplD // rplV</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>negative regulation of macromolecule biosynthetic process</t>
+        </is>
+      </c>
+      <c r="K121" s="1" t="n">
+        <v>0.08139449999999999</v>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>rplJ // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>negative regulation of biosynthetic process</t>
+        </is>
+      </c>
+      <c r="K122" s="1" t="n">
+        <v>0.08198388</v>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>rplJ // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>primary metabolic process</t>
+        </is>
+      </c>
+      <c r="K123" s="1" t="n">
+        <v>0.08317098000000001</v>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>rplJ // truB // phoR // rplV // rplD // tufB</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>protein phosphorylation</t>
+        </is>
+      </c>
+      <c r="K124" s="1" t="n">
+        <v>0.08507172</v>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>fis</t>
+        </is>
+      </c>
+      <c r="K125" s="1" t="n">
+        <v>0.08555052</v>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>tufB // truB</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>protein kinase activity</t>
+        </is>
+      </c>
+      <c r="K126" s="1" t="n">
+        <v>0.08692796999999999</v>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>inorganic anion transport</t>
+        </is>
+      </c>
+      <c r="K127" s="1" t="n">
+        <v>0.08692796999999999</v>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>cellular response to starvation</t>
+        </is>
+      </c>
+      <c r="K128" s="1" t="n">
+        <v>0.09063045</v>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>negative regulation of macromolecule metabolic process</t>
+        </is>
+      </c>
+      <c r="K129" s="1" t="n">
+        <v>0.09099575999999999</v>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>rplJ // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>negative regulation of metabolic process</t>
+        </is>
+      </c>
+      <c r="K130" s="1" t="n">
+        <v>0.09222093000000001</v>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>rplJ // rplD</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>cellular response to nutrient levels</t>
+        </is>
+      </c>
+      <c r="K131" s="1" t="n">
+        <v>0.09615914</v>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>phoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>protein-RNA complex assembly</t>
+        </is>
+      </c>
+      <c r="K132" s="1" t="n">
+        <v>0.09615914</v>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>rplV</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>protein-RNA complex organization</t>
+        </is>
+      </c>
+      <c r="K133" s="1" t="n">
+        <v>0.09615914</v>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>rplV</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>enzyme regulator activity</t>
+        </is>
+      </c>
+      <c r="K134" s="1" t="n">
+        <v>0.097995386</v>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>rplD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>